<commit_message>
fixed hurricane and poison controlled by cleanse tag
</commit_message>
<xml_diff>
--- a/nettux-new-mons.xlsx
+++ b/nettux-new-mons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lewis\pokeemerald-nettux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDA6A84-50A2-4DF6-9AC1-18B717B8FFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF8620F-D548-4B04-A15E-00E943D0FD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1605" yWindow="1335" windowWidth="10485" windowHeight="11385" xr2:uid="{4D0F1F34-F3E4-433F-B9BC-51AD106AAB02}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{4D0F1F34-F3E4-433F-B9BC-51AD106AAB02}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Dex" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2108" uniqueCount="1409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="1418">
   <si>
     <t>Sandshrew</t>
   </si>
@@ -3990,9 +3990,6 @@
     <t>Route110 Fishing</t>
   </si>
   <si>
-    <t>GraniteCave_1F, GraniteCave_B2F</t>
-  </si>
-  <si>
     <t>Poltchageist</t>
   </si>
   <si>
@@ -4038,9 +4035,6 @@
     <t>Route 101, Route103</t>
   </si>
   <si>
-    <t xml:space="preserve">, , </t>
-  </si>
-  <si>
     <t>Route104, , GraniteCave_B2F</t>
   </si>
   <si>
@@ -4068,9 +4062,6 @@
     <t xml:space="preserve">Route104, , </t>
   </si>
   <si>
-    <t>Route103, GraniteCave_1F</t>
-  </si>
-  <si>
     <t>Doduo</t>
   </si>
   <si>
@@ -4122,9 +4113,6 @@
     <t>Clodsire</t>
   </si>
   <si>
-    <t>Route 117, MauvilleCity</t>
-  </si>
-  <si>
     <t xml:space="preserve">GraniteCave_1F, , , </t>
   </si>
   <si>
@@ -4134,9 +4122,6 @@
     <t xml:space="preserve">, GraniteCave_B2F, </t>
   </si>
   <si>
-    <t>, , Route117</t>
-  </si>
-  <si>
     <t>GraniteCave_B2F, GraniteCave_Steven</t>
   </si>
   <si>
@@ -4170,9 +4155,6 @@
     <t>Route104, MeteorFalls_1F_1R</t>
   </si>
   <si>
-    <t>Route104, GraniteCave_1F, MeteorFalls_1F_1R</t>
-  </si>
-  <si>
     <t>GraniteCave_B1F, MeteorFalls_1F_1R</t>
   </si>
   <si>
@@ -4257,13 +4239,58 @@
     <t>MeteorFalls_1F_1R, MtChimney</t>
   </si>
   <si>
-    <t>Route112, MtChimney</t>
-  </si>
-  <si>
     <t>MtChimney</t>
   </si>
   <si>
     <t>FieryPath, Route113, MtChimney</t>
+  </si>
+  <si>
+    <t>Route113, Route111</t>
+  </si>
+  <si>
+    <t>MeteorFalls_1F_1R, MtChimney, Route111</t>
+  </si>
+  <si>
+    <t>RusturfTunnel, Route111</t>
+  </si>
+  <si>
+    <t>MtChimney, Route111</t>
+  </si>
+  <si>
+    <t>Route112, Route111</t>
+  </si>
+  <si>
+    <t>GraniteCave_1F, GraniteCave_B2F, Route111</t>
+  </si>
+  <si>
+    <t>Route111</t>
+  </si>
+  <si>
+    <t>Route 117, MauvilleCity, Route111</t>
+  </si>
+  <si>
+    <t>Route103, GraniteCave_1F, MirageTower</t>
+  </si>
+  <si>
+    <t>MirageTower</t>
+  </si>
+  <si>
+    <t>Route113, Route111, MirageTower</t>
+  </si>
+  <si>
+    <t>GraniteCave_B1F, Route111, MirageTower</t>
+  </si>
+  <si>
+    <t>Route117, MirageTower</t>
+  </si>
+  <si>
+    <t>Route104, GraniteCave_1F, MeteorFalls_1F_1R, MirageTower</t>
+  </si>
+  <si>
+    <t>MeteorFalls_1F_1R, MirageTower</t>
+  </si>
+  <si>
+    <t>Route112, MtChimney, MirageTower</t>
   </si>
 </sst>
 </file>
@@ -4697,7 +4724,7 @@
         <v>315</v>
       </c>
       <c r="C2" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="D2" t="s">
         <v>318</v>
@@ -4795,7 +4822,7 @@
         <v>168</v>
       </c>
       <c r="C9" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
       <c r="D9" t="s">
         <v>256</v>
@@ -4809,7 +4836,7 @@
         <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
       <c r="D10" t="s">
         <v>256</v>
@@ -4837,7 +4864,7 @@
         <v>241</v>
       </c>
       <c r="C12" t="s">
-        <v>1403</v>
+        <v>1397</v>
       </c>
       <c r="D12" t="s">
         <v>265</v>
@@ -4851,7 +4878,7 @@
         <v>158</v>
       </c>
       <c r="C13" t="s">
-        <v>1351</v>
+        <v>1348</v>
       </c>
       <c r="D13" t="s">
         <v>274</v>
@@ -4876,7 +4903,7 @@
         <v>165</v>
       </c>
       <c r="C15" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="D15" t="s">
         <v>220</v>
@@ -4890,7 +4917,7 @@
         <v>221</v>
       </c>
       <c r="C16" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D16" t="s">
         <v>220</v>
@@ -4904,7 +4931,7 @@
         <v>184</v>
       </c>
       <c r="C17" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="D17" t="s">
         <v>220</v>
@@ -4943,7 +4970,7 @@
         <v>156</v>
       </c>
       <c r="C20" t="s">
-        <v>1382</v>
+        <v>1376</v>
       </c>
       <c r="D20" t="s">
         <v>278</v>
@@ -4957,7 +4984,7 @@
         <v>160</v>
       </c>
       <c r="C21" t="s">
-        <v>1371</v>
+        <v>1406</v>
       </c>
       <c r="D21" t="s">
         <v>299</v>
@@ -4982,7 +5009,7 @@
         <v>188</v>
       </c>
       <c r="C23" t="s">
-        <v>1380</v>
+        <v>1374</v>
       </c>
       <c r="D23" t="s">
         <v>224</v>
@@ -4996,7 +5023,7 @@
         <v>149</v>
       </c>
       <c r="C24" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D24" t="s">
         <v>224</v>
@@ -5021,7 +5048,7 @@
         <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>1379</v>
+        <v>1373</v>
       </c>
       <c r="D26" t="s">
         <v>276</v>
@@ -5035,7 +5062,7 @@
         <v>117</v>
       </c>
       <c r="C27" t="s">
-        <v>1379</v>
+        <v>1373</v>
       </c>
       <c r="D27" t="s">
         <v>226</v>
@@ -5049,7 +5076,7 @@
         <v>47</v>
       </c>
       <c r="C28" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="D28" t="s">
         <v>226</v>
@@ -5063,7 +5090,7 @@
         <v>134</v>
       </c>
       <c r="C29" t="s">
-        <v>1371</v>
+        <v>1406</v>
       </c>
       <c r="D29" t="s">
         <v>226</v>
@@ -5099,7 +5126,7 @@
         <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>1366</v>
+        <v>1361</v>
       </c>
       <c r="D32" t="s">
         <v>689</v>
@@ -5113,7 +5140,7 @@
         <v>229</v>
       </c>
       <c r="C33" t="s">
-        <v>1294</v>
+        <v>1404</v>
       </c>
       <c r="D33" t="s">
         <v>258</v>
@@ -5141,7 +5168,7 @@
         <v>327</v>
       </c>
       <c r="C35" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
       <c r="D35" t="s">
         <v>323</v>
@@ -5222,7 +5249,7 @@
         <v>280</v>
       </c>
       <c r="C41" t="s">
-        <v>1379</v>
+        <v>1373</v>
       </c>
       <c r="D41" t="s">
         <v>277</v>
@@ -5291,7 +5318,7 @@
         <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>1407</v>
+        <v>1400</v>
       </c>
       <c r="D47" t="s">
         <v>264</v>
@@ -5333,7 +5360,7 @@
         <v>200</v>
       </c>
       <c r="C50" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="D50" t="s">
         <v>266</v>
@@ -5358,7 +5385,7 @@
         <v>196</v>
       </c>
       <c r="C52" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D52" t="s">
         <v>266</v>
@@ -5372,7 +5399,7 @@
         <v>203</v>
       </c>
       <c r="C53" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="D53" t="s">
         <v>209</v>
@@ -5386,7 +5413,7 @@
         <v>124</v>
       </c>
       <c r="C54" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="D54" t="s">
         <v>209</v>
@@ -5400,7 +5427,7 @@
         <v>207</v>
       </c>
       <c r="C55" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="D55" t="s">
         <v>228</v>
@@ -5414,7 +5441,7 @@
         <v>125</v>
       </c>
       <c r="C56" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="D56" t="s">
         <v>228</v>
@@ -5428,7 +5455,7 @@
         <v>113</v>
       </c>
       <c r="C57" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
       <c r="D57" t="s">
         <v>216</v>
@@ -5442,7 +5469,7 @@
         <v>116</v>
       </c>
       <c r="C58" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="D58" t="s">
         <v>216</v>
@@ -5456,7 +5483,7 @@
         <v>127</v>
       </c>
       <c r="C59" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="D59" t="s">
         <v>215</v>
@@ -5470,7 +5497,7 @@
         <v>128</v>
       </c>
       <c r="C60" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="D60" t="s">
         <v>231</v>
@@ -5484,7 +5511,7 @@
         <v>111</v>
       </c>
       <c r="C61" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="D61" t="s">
         <v>210</v>
@@ -5498,7 +5525,7 @@
         <v>112</v>
       </c>
       <c r="C62" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="D62" t="s">
         <v>210</v>
@@ -5612,7 +5639,7 @@
         <v>139</v>
       </c>
       <c r="C71" t="s">
-        <v>1406</v>
+        <v>1417</v>
       </c>
       <c r="D71" t="s">
         <v>259</v>
@@ -5640,7 +5667,7 @@
         <v>50</v>
       </c>
       <c r="C73" t="s">
-        <v>1381</v>
+        <v>1375</v>
       </c>
       <c r="D73" t="s">
         <v>301</v>
@@ -5698,7 +5725,7 @@
         <v>172</v>
       </c>
       <c r="C78" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D78" t="s">
         <v>284</v>
@@ -5748,7 +5775,7 @@
         <v>288</v>
       </c>
       <c r="C82" t="s">
-        <v>1372</v>
+        <v>1402</v>
       </c>
       <c r="D82" t="s">
         <v>289</v>
@@ -5773,7 +5800,7 @@
         <v>204</v>
       </c>
       <c r="C84" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D84" t="s">
         <v>293</v>
@@ -5875,7 +5902,7 @@
         <v>83</v>
       </c>
       <c r="C93" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="D93" t="s">
         <v>273</v>
@@ -5977,7 +6004,7 @@
         <v>192</v>
       </c>
       <c r="C102" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="D102" t="s">
         <v>214</v>
@@ -5991,7 +6018,7 @@
         <v>105</v>
       </c>
       <c r="C103" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="D103" t="s">
         <v>214</v>
@@ -6005,7 +6032,7 @@
         <v>171</v>
       </c>
       <c r="C104" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="D104" t="s">
         <v>225</v>
@@ -6019,7 +6046,7 @@
         <v>169</v>
       </c>
       <c r="C105" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D105" t="s">
         <v>212</v>
@@ -6033,7 +6060,7 @@
         <v>103</v>
       </c>
       <c r="C106" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D106" t="s">
         <v>219</v>
@@ -6047,7 +6074,7 @@
         <v>213</v>
       </c>
       <c r="C107" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
       <c r="D107" t="s">
         <v>251</v>
@@ -6075,7 +6102,7 @@
         <v>102</v>
       </c>
       <c r="C109" t="s">
-        <v>1390</v>
+        <v>1384</v>
       </c>
       <c r="D109" t="s">
         <v>211</v>
@@ -6136,7 +6163,7 @@
         <v>106</v>
       </c>
       <c r="C114" t="s">
-        <v>1386</v>
+        <v>1380</v>
       </c>
       <c r="D114" t="s">
         <v>232</v>
@@ -6150,7 +6177,7 @@
         <v>189</v>
       </c>
       <c r="C115" t="s">
-        <v>1376</v>
+        <v>1371</v>
       </c>
       <c r="D115" t="s">
         <v>236</v>
@@ -6192,7 +6219,7 @@
         <v>237</v>
       </c>
       <c r="C118" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="D118" t="s">
         <v>235</v>
@@ -6250,7 +6277,7 @@
         <v>141</v>
       </c>
       <c r="C123" t="s">
-        <v>1401</v>
+        <v>1395</v>
       </c>
       <c r="D123" t="s">
         <v>269</v>
@@ -6264,7 +6291,7 @@
         <v>175</v>
       </c>
       <c r="C124" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="D124" t="s">
         <v>261</v>
@@ -6325,7 +6352,7 @@
         <v>182</v>
       </c>
       <c r="C129" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="D129" t="s">
         <v>248</v>
@@ -6361,7 +6388,7 @@
         <v>179</v>
       </c>
       <c r="C132" t="s">
-        <v>1370</v>
+        <v>1365</v>
       </c>
       <c r="D132" t="s">
         <v>268</v>
@@ -6375,7 +6402,7 @@
         <v>240</v>
       </c>
       <c r="C133" t="s">
-        <v>1347</v>
+        <v>1344</v>
       </c>
       <c r="D133" t="s">
         <v>247</v>
@@ -6436,7 +6463,7 @@
         <v>243</v>
       </c>
       <c r="C138" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="D138" t="s">
         <v>290</v>
@@ -6464,7 +6491,7 @@
         <v>76</v>
       </c>
       <c r="C140" t="s">
-        <v>1391</v>
+        <v>1385</v>
       </c>
       <c r="D140" t="s">
         <v>297</v>
@@ -6478,7 +6505,7 @@
         <v>170</v>
       </c>
       <c r="C141" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="D141" t="s">
         <v>285</v>
@@ -6723,7 +6750,7 @@
         <v>28</v>
       </c>
       <c r="C163" t="s">
-        <v>1389</v>
+        <v>1383</v>
       </c>
       <c r="D163" t="s">
         <v>302</v>
@@ -6751,7 +6778,7 @@
         <v>316</v>
       </c>
       <c r="C165" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="D165" t="s">
         <v>318</v>
@@ -6765,7 +6792,7 @@
         <v>326</v>
       </c>
       <c r="C166" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="D166" t="s">
         <v>325</v>
@@ -6779,7 +6806,7 @@
         <v>328</v>
       </c>
       <c r="C167" t="s">
-        <v>1379</v>
+        <v>1373</v>
       </c>
       <c r="D167" t="s">
         <v>325</v>
@@ -6793,7 +6820,7 @@
         <v>329</v>
       </c>
       <c r="C168" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="D168" t="s">
         <v>325</v>
@@ -6807,7 +6834,7 @@
         <v>333</v>
       </c>
       <c r="C169" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="D169" t="s">
         <v>325</v>
@@ -6821,7 +6848,7 @@
         <v>342</v>
       </c>
       <c r="C170" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="D170" t="s">
         <v>325</v>
@@ -6835,7 +6862,7 @@
         <v>343</v>
       </c>
       <c r="C171" t="s">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="D171" t="s">
         <v>325</v>
@@ -6997,7 +7024,7 @@
         <v>155</v>
       </c>
       <c r="C183" t="s">
-        <v>1358</v>
+        <v>1355</v>
       </c>
       <c r="D183" t="s">
         <v>217</v>
@@ -7022,7 +7049,7 @@
         <v>152</v>
       </c>
       <c r="C185" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
       <c r="D185" t="s">
         <v>217</v>
@@ -7036,7 +7063,7 @@
         <v>162</v>
       </c>
       <c r="C186" t="s">
-        <v>1368</v>
+        <v>1363</v>
       </c>
       <c r="D186" t="s">
         <v>222</v>
@@ -7152,7 +7179,7 @@
         <v>373</v>
       </c>
       <c r="C199" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
@@ -7179,7 +7206,7 @@
         <v>376</v>
       </c>
       <c r="C202" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -7214,7 +7241,7 @@
         <v>380</v>
       </c>
       <c r="C206" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -7225,7 +7252,7 @@
         <v>381</v>
       </c>
       <c r="C207" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
@@ -7255,7 +7282,7 @@
         <v>0</v>
       </c>
       <c r="C210" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
@@ -7274,7 +7301,7 @@
         <v>386</v>
       </c>
       <c r="C212" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
@@ -7285,7 +7312,7 @@
         <v>387</v>
       </c>
       <c r="C213" t="s">
-        <v>1361</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
@@ -7304,7 +7331,7 @@
         <v>389</v>
       </c>
       <c r="C215" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -7315,7 +7342,7 @@
         <v>390</v>
       </c>
       <c r="C216" t="s">
-        <v>1361</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
@@ -7353,7 +7380,7 @@
         <v>1</v>
       </c>
       <c r="C220" t="s">
-        <v>1352</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
@@ -7391,7 +7418,7 @@
         <v>398</v>
       </c>
       <c r="C224" t="s">
-        <v>1377</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
@@ -7402,7 +7429,7 @@
         <v>399</v>
       </c>
       <c r="C225" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
@@ -7440,7 +7467,7 @@
         <v>405</v>
       </c>
       <c r="C229" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
@@ -7475,7 +7502,7 @@
         <v>409</v>
       </c>
       <c r="C233" t="s">
-        <v>1333</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -7510,7 +7537,7 @@
         <v>413</v>
       </c>
       <c r="C237" t="s">
-        <v>1384</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
@@ -7529,7 +7556,7 @@
         <v>415</v>
       </c>
       <c r="C239" t="s">
-        <v>1385</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
@@ -7548,7 +7575,7 @@
         <v>418</v>
       </c>
       <c r="C241" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
@@ -7567,7 +7594,7 @@
         <v>420</v>
       </c>
       <c r="C243" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
@@ -7594,7 +7621,7 @@
         <v>424</v>
       </c>
       <c r="C246" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
@@ -7624,7 +7651,7 @@
         <v>427</v>
       </c>
       <c r="C249" t="s">
-        <v>1385</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
@@ -7686,7 +7713,7 @@
         <v>433</v>
       </c>
       <c r="C256" t="s">
-        <v>1404</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
@@ -7713,7 +7740,7 @@
         <v>435</v>
       </c>
       <c r="C259" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
@@ -7770,7 +7797,7 @@
         <v>440</v>
       </c>
       <c r="C265" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
@@ -7778,7 +7805,7 @@
         <v>797</v>
       </c>
       <c r="B266" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
@@ -7813,7 +7840,7 @@
         <v>445</v>
       </c>
       <c r="C270" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
@@ -7848,7 +7875,7 @@
         <v>449</v>
       </c>
       <c r="C274" t="s">
-        <v>1364</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
@@ -7875,7 +7902,7 @@
         <v>452</v>
       </c>
       <c r="C277" t="s">
-        <v>1402</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
@@ -7905,7 +7932,7 @@
         <v>456</v>
       </c>
       <c r="C280" t="s">
-        <v>1379</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
@@ -7940,7 +7967,7 @@
         <v>460</v>
       </c>
       <c r="C284" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
@@ -7959,7 +7986,7 @@
         <v>462</v>
       </c>
       <c r="C286" t="s">
-        <v>1365</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
@@ -7978,7 +8005,7 @@
         <v>465</v>
       </c>
       <c r="C288" t="s">
-        <v>1386</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
@@ -7989,7 +8016,7 @@
         <v>466</v>
       </c>
       <c r="C289" t="s">
-        <v>1386</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
@@ -8032,7 +8059,7 @@
         <v>472</v>
       </c>
       <c r="C294" t="s">
-        <v>1402</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
@@ -8067,7 +8094,7 @@
         <v>480</v>
       </c>
       <c r="C298" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
@@ -8110,7 +8137,7 @@
         <v>8</v>
       </c>
       <c r="C303" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
@@ -8129,7 +8156,7 @@
         <v>487</v>
       </c>
       <c r="C305" t="s">
-        <v>1367</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -8140,7 +8167,7 @@
         <v>489</v>
       </c>
       <c r="C306" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
@@ -8167,7 +8194,7 @@
         <v>10</v>
       </c>
       <c r="C309" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
@@ -8265,6 +8292,9 @@
       <c r="B321" t="s">
         <v>515</v>
       </c>
+      <c r="C321" t="s">
+        <v>1411</v>
+      </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
@@ -8282,7 +8312,7 @@
         <v>517</v>
       </c>
       <c r="C323" t="s">
-        <v>1405</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
@@ -8301,7 +8331,7 @@
         <v>519</v>
       </c>
       <c r="C325" t="s">
-        <v>1405</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
@@ -8448,7 +8478,7 @@
         <v>50</v>
       </c>
       <c r="C343" t="s">
-        <v>1379</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
@@ -8523,7 +8553,7 @@
         <v>12</v>
       </c>
       <c r="C352" t="s">
-        <v>1369</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.25">
@@ -8542,7 +8572,7 @@
         <v>538</v>
       </c>
       <c r="C354" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.25">
@@ -8577,7 +8607,7 @@
         <v>543</v>
       </c>
       <c r="C358" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.25">
@@ -8604,7 +8634,7 @@
         <v>547</v>
       </c>
       <c r="C361" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
@@ -8639,7 +8669,7 @@
         <v>549</v>
       </c>
       <c r="C365" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
@@ -8666,7 +8696,7 @@
         <v>554</v>
       </c>
       <c r="C368" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.25">
@@ -8677,7 +8707,7 @@
         <v>556</v>
       </c>
       <c r="C369" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.25">
@@ -8704,7 +8734,7 @@
         <v>559</v>
       </c>
       <c r="C372" t="s">
-        <v>1311</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.25">
@@ -8758,7 +8788,7 @@
         <v>565</v>
       </c>
       <c r="C378" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="379" spans="1:3" x14ac:dyDescent="0.25">
@@ -8769,7 +8799,7 @@
         <v>566</v>
       </c>
       <c r="C379" t="s">
-        <v>1388</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.25">
@@ -8807,7 +8837,7 @@
         <v>572</v>
       </c>
       <c r="C383" t="s">
-        <v>1408</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.25">
@@ -8925,7 +8955,7 @@
         <v>464</v>
       </c>
       <c r="C397" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.25">
@@ -8936,7 +8966,7 @@
         <v>467</v>
       </c>
       <c r="C398" t="s">
-        <v>1386</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.25">
@@ -9083,7 +9113,7 @@
         <v>597</v>
       </c>
       <c r="C416" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.25">
@@ -9151,7 +9181,7 @@
         <v>603</v>
       </c>
       <c r="C423" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.25">
@@ -9170,7 +9200,7 @@
         <v>605</v>
       </c>
       <c r="C425" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.25">
@@ -9189,7 +9219,7 @@
         <v>104</v>
       </c>
       <c r="C427" t="s">
-        <v>1367</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="428" spans="1:3" x14ac:dyDescent="0.25">
@@ -9259,7 +9289,7 @@
         <v>612</v>
       </c>
       <c r="C435" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="436" spans="1:3" x14ac:dyDescent="0.25">
@@ -9286,7 +9316,7 @@
         <v>615</v>
       </c>
       <c r="C438" t="s">
-        <v>1387</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.25">
@@ -9312,6 +9342,9 @@
       <c r="B441" t="s">
         <v>617</v>
       </c>
+      <c r="C441" t="s">
+        <v>1411</v>
+      </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
@@ -9356,7 +9389,7 @@
         <v>622</v>
       </c>
       <c r="C446" t="s">
-        <v>1392</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
@@ -9469,7 +9502,7 @@
         <v>635</v>
       </c>
       <c r="C459" t="s">
-        <v>1372</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.25">
@@ -9512,7 +9545,7 @@
         <v>640</v>
       </c>
       <c r="C464" t="s">
-        <v>1375</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
@@ -9531,7 +9564,7 @@
         <v>642</v>
       </c>
       <c r="C466" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
@@ -9542,7 +9575,7 @@
         <v>643</v>
       </c>
       <c r="C467" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
@@ -9553,7 +9586,7 @@
         <v>644</v>
       </c>
       <c r="C468" t="s">
-        <v>1378</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
@@ -9564,7 +9597,7 @@
         <v>645</v>
       </c>
       <c r="C469" t="s">
-        <v>1378</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="470" spans="1:3" x14ac:dyDescent="0.25">
@@ -9594,7 +9627,7 @@
         <v>648</v>
       </c>
       <c r="C472" t="s">
-        <v>1384</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
@@ -9613,7 +9646,7 @@
         <v>650</v>
       </c>
       <c r="C474" t="s">
-        <v>1306</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
@@ -9854,7 +9887,7 @@
         <v>674</v>
       </c>
       <c r="C503" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
@@ -9993,7 +10026,7 @@
         <v>136</v>
       </c>
       <c r="C520" t="s">
-        <v>1343</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
@@ -10012,7 +10045,7 @@
         <v>107</v>
       </c>
       <c r="C522" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
@@ -10360,7 +10393,7 @@
         <v>153</v>
       </c>
       <c r="C564" t="s">
-        <v>1317</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="565" spans="1:3" x14ac:dyDescent="0.25">
@@ -10395,7 +10428,7 @@
         <v>79</v>
       </c>
       <c r="C568" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="569" spans="1:3" x14ac:dyDescent="0.25">
@@ -10513,7 +10546,7 @@
         <v>65</v>
       </c>
       <c r="C582" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="583" spans="1:3" x14ac:dyDescent="0.25">
@@ -10524,7 +10557,7 @@
         <v>66</v>
       </c>
       <c r="C583" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="584" spans="1:3" x14ac:dyDescent="0.25">
@@ -10551,7 +10584,7 @@
         <v>72</v>
       </c>
       <c r="C586" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="587" spans="1:3" x14ac:dyDescent="0.25">
@@ -10748,7 +10781,7 @@
     </row>
     <row r="611" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B611" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="C611" t="s">
         <v>1307</v>
@@ -10756,12 +10789,12 @@
     </row>
     <row r="612" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B612" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="613" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B613" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="C613" t="s">
         <v>1306</v>
@@ -10769,7 +10802,7 @@
     </row>
     <row r="614" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B614" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="C614" t="s">
         <v>1295</v>
@@ -10777,7 +10810,7 @@
     </row>
     <row r="615" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B615" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="C615" t="s">
         <v>1294</v>
@@ -10785,105 +10818,108 @@
     </row>
     <row r="616" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B616" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="617" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B617" t="s">
-        <v>1348</v>
+        <v>1345</v>
       </c>
       <c r="C617" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="618" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B618" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="619" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B619" t="s">
-        <v>1354</v>
+        <v>1351</v>
       </c>
       <c r="C619" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="620" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B620" t="s">
-        <v>1355</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="621" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B621" t="s">
-        <v>1356</v>
+        <v>1353</v>
       </c>
       <c r="C621" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="622" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B622" t="s">
-        <v>1357</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="623" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B623" t="s">
-        <v>1359</v>
+        <v>1356</v>
       </c>
       <c r="C623" t="s">
-        <v>1374</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="624" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B624" t="s">
-        <v>1360</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="625" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B625" t="s">
-        <v>1393</v>
+        <v>1387</v>
       </c>
       <c r="C625" t="s">
-        <v>1407</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="626" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B626" t="s">
-        <v>1394</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="627" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B627" t="s">
-        <v>1395</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="628" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B628" t="s">
-        <v>1396</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="629" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B629" t="s">
-        <v>1397</v>
+        <v>1391</v>
       </c>
       <c r="C629" t="s">
-        <v>1407</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="630" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B630" t="s">
-        <v>1398</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="631" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B631" t="s">
-        <v>1399</v>
+        <v>1393</v>
+      </c>
+      <c r="C631" t="s">
+        <v>1408</v>
       </c>
     </row>
     <row r="632" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B632" t="s">
-        <v>1400</v>
+        <v>1394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added elite 4 teams, blackout and acid rain weather
</commit_message>
<xml_diff>
--- a/nettux-new-mons.xlsx
+++ b/nettux-new-mons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lewis\pokeemerald-nettux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF8620F-D548-4B04-A15E-00E943D0FD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A36E52C9-B54A-4FDD-BA3D-B6E545F8772D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{4D0F1F34-F3E4-433F-B9BC-51AD106AAB02}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="12480" windowHeight="15585" xr2:uid="{4D0F1F34-F3E4-433F-B9BC-51AD106AAB02}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Dex" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="1418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2139" uniqueCount="1439">
   <si>
     <t>Sandshrew</t>
   </si>
@@ -4023,9 +4023,6 @@
     <t>Route 102, Route103</t>
   </si>
   <si>
-    <t>Route 102, Route103, Route104</t>
-  </si>
-  <si>
     <t>Route103</t>
   </si>
   <si>
@@ -4035,9 +4032,6 @@
     <t>Route 101, Route103</t>
   </si>
   <si>
-    <t>Route104, , GraniteCave_B2F</t>
-  </si>
-  <si>
     <t>Route 102, PetalburgWoods</t>
   </si>
   <si>
@@ -4236,18 +4230,12 @@
     <t>Route 117, MtChimney</t>
   </si>
   <si>
-    <t>MeteorFalls_1F_1R, MtChimney</t>
-  </si>
-  <si>
     <t>MtChimney</t>
   </si>
   <si>
     <t>FieryPath, Route113, MtChimney</t>
   </si>
   <si>
-    <t>Route113, Route111</t>
-  </si>
-  <si>
     <t>MeteorFalls_1F_1R, MtChimney, Route111</t>
   </si>
   <si>
@@ -4263,15 +4251,9 @@
     <t>GraniteCave_1F, GraniteCave_B2F, Route111</t>
   </si>
   <si>
-    <t>Route111</t>
-  </si>
-  <si>
     <t>Route 117, MauvilleCity, Route111</t>
   </si>
   <si>
-    <t>Route103, GraniteCave_1F, MirageTower</t>
-  </si>
-  <si>
     <t>MirageTower</t>
   </si>
   <si>
@@ -4291,6 +4273,87 @@
   </si>
   <si>
     <t>Route112, MtChimney, MirageTower</t>
+  </si>
+  <si>
+    <t>Route 102, Route103, Route104, Route118 Surf</t>
+  </si>
+  <si>
+    <t>Route118 Surf</t>
+  </si>
+  <si>
+    <t>Route 101, Route 102, Route104, Route118 Surf</t>
+  </si>
+  <si>
+    <t>Route110, Route118, Route118 Surf</t>
+  </si>
+  <si>
+    <t>Route110, Route118</t>
+  </si>
+  <si>
+    <t>Route118</t>
+  </si>
+  <si>
+    <t>Route111, Route118</t>
+  </si>
+  <si>
+    <t>Route113, Route111, Route118</t>
+  </si>
+  <si>
+    <t>MeteorFalls_1F_1R, Route118</t>
+  </si>
+  <si>
+    <t>MeteorFalls_1F_1R, MtChimney, Route118</t>
+  </si>
+  <si>
+    <t>MirageTower, Route118</t>
+  </si>
+  <si>
+    <t>Route118 Fishing, Route119 Fishing</t>
+  </si>
+  <si>
+    <t>Route103, GraniteCave_1F, MirageTower, Route118 Fishing, Route119 Fishing</t>
+  </si>
+  <si>
+    <t>Route106 Fishing, Route118 Fishing, Route119 Fishing</t>
+  </si>
+  <si>
+    <t>Zigzagoon Galar</t>
+  </si>
+  <si>
+    <t>Linoone Galar</t>
+  </si>
+  <si>
+    <t>Obstagoon</t>
+  </si>
+  <si>
+    <t>Route 119</t>
+  </si>
+  <si>
+    <t>RusturfTunnel, Route 119</t>
+  </si>
+  <si>
+    <t>MauvilleCity, Route 119</t>
+  </si>
+  <si>
+    <t>MeteorFalls_1F_1R, Route 119</t>
+  </si>
+  <si>
+    <t>Route120</t>
+  </si>
+  <si>
+    <t>Route 119, Route120</t>
+  </si>
+  <si>
+    <t>Route104, GraniteCave_B2F, Route120</t>
+  </si>
+  <si>
+    <t>Route112, Route111, Route120</t>
+  </si>
+  <si>
+    <t>Route112, Route120</t>
+  </si>
+  <si>
+    <t>PetalburgWoods, Route120</t>
   </si>
 </sst>
 </file>
@@ -4693,7 +4756,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D266181C-CB66-47C1-88A5-38F785E7523D}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D632"/>
+  <dimension ref="A1:D635"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
@@ -4724,7 +4787,7 @@
         <v>315</v>
       </c>
       <c r="C2" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D2" t="s">
         <v>318</v>
@@ -4822,7 +4885,7 @@
         <v>168</v>
       </c>
       <c r="C9" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="D9" t="s">
         <v>256</v>
@@ -4836,7 +4899,7 @@
         <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="D10" t="s">
         <v>256</v>
@@ -4864,7 +4927,7 @@
         <v>241</v>
       </c>
       <c r="C12" t="s">
-        <v>1397</v>
+        <v>1395</v>
       </c>
       <c r="D12" t="s">
         <v>265</v>
@@ -4878,7 +4941,7 @@
         <v>158</v>
       </c>
       <c r="C13" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="D13" t="s">
         <v>274</v>
@@ -4903,7 +4966,7 @@
         <v>165</v>
       </c>
       <c r="C15" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="D15" t="s">
         <v>220</v>
@@ -4917,7 +4980,7 @@
         <v>221</v>
       </c>
       <c r="C16" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="D16" t="s">
         <v>220</v>
@@ -4931,7 +4994,7 @@
         <v>184</v>
       </c>
       <c r="C17" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="D17" t="s">
         <v>220</v>
@@ -4970,7 +5033,7 @@
         <v>156</v>
       </c>
       <c r="C20" t="s">
-        <v>1376</v>
+        <v>1374</v>
       </c>
       <c r="D20" t="s">
         <v>278</v>
@@ -4984,7 +5047,7 @@
         <v>160</v>
       </c>
       <c r="C21" t="s">
-        <v>1406</v>
+        <v>1436</v>
       </c>
       <c r="D21" t="s">
         <v>299</v>
@@ -5009,7 +5072,7 @@
         <v>188</v>
       </c>
       <c r="C23" t="s">
-        <v>1374</v>
+        <v>1372</v>
       </c>
       <c r="D23" t="s">
         <v>224</v>
@@ -5023,7 +5086,7 @@
         <v>149</v>
       </c>
       <c r="C24" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="D24" t="s">
         <v>224</v>
@@ -5048,7 +5111,7 @@
         <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="D26" t="s">
         <v>276</v>
@@ -5062,7 +5125,7 @@
         <v>117</v>
       </c>
       <c r="C27" t="s">
-        <v>1373</v>
+        <v>1432</v>
       </c>
       <c r="D27" t="s">
         <v>226</v>
@@ -5076,7 +5139,7 @@
         <v>47</v>
       </c>
       <c r="C28" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="D28" t="s">
         <v>226</v>
@@ -5090,7 +5153,7 @@
         <v>134</v>
       </c>
       <c r="C29" t="s">
-        <v>1406</v>
+        <v>1402</v>
       </c>
       <c r="D29" t="s">
         <v>226</v>
@@ -5126,7 +5189,7 @@
         <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>1361</v>
+        <v>1359</v>
       </c>
       <c r="D32" t="s">
         <v>689</v>
@@ -5140,7 +5203,7 @@
         <v>229</v>
       </c>
       <c r="C33" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="D33" t="s">
         <v>258</v>
@@ -5168,7 +5231,7 @@
         <v>327</v>
       </c>
       <c r="C35" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="D35" t="s">
         <v>323</v>
@@ -5249,7 +5312,7 @@
         <v>280</v>
       </c>
       <c r="C41" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="D41" t="s">
         <v>277</v>
@@ -5318,7 +5381,7 @@
         <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
       <c r="D47" t="s">
         <v>264</v>
@@ -5332,7 +5395,7 @@
         <v>199</v>
       </c>
       <c r="C48" t="s">
-        <v>1294</v>
+        <v>1430</v>
       </c>
       <c r="D48" t="s">
         <v>266</v>
@@ -5346,7 +5409,7 @@
         <v>198</v>
       </c>
       <c r="C49" t="s">
-        <v>1294</v>
+        <v>1430</v>
       </c>
       <c r="D49" t="s">
         <v>266</v>
@@ -5360,7 +5423,7 @@
         <v>200</v>
       </c>
       <c r="C50" t="s">
-        <v>1350</v>
+        <v>1431</v>
       </c>
       <c r="D50" t="s">
         <v>266</v>
@@ -5385,7 +5448,7 @@
         <v>196</v>
       </c>
       <c r="C52" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="D52" t="s">
         <v>266</v>
@@ -5399,7 +5462,7 @@
         <v>203</v>
       </c>
       <c r="C53" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="D53" t="s">
         <v>209</v>
@@ -5441,7 +5504,7 @@
         <v>125</v>
       </c>
       <c r="C56" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="D56" t="s">
         <v>228</v>
@@ -5455,7 +5518,7 @@
         <v>113</v>
       </c>
       <c r="C57" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="D57" t="s">
         <v>216</v>
@@ -5525,7 +5588,7 @@
         <v>112</v>
       </c>
       <c r="C62" t="s">
-        <v>1324</v>
+        <v>1414</v>
       </c>
       <c r="D62" t="s">
         <v>210</v>
@@ -5639,7 +5702,7 @@
         <v>139</v>
       </c>
       <c r="C71" t="s">
-        <v>1417</v>
+        <v>1411</v>
       </c>
       <c r="D71" t="s">
         <v>259</v>
@@ -5667,7 +5730,7 @@
         <v>50</v>
       </c>
       <c r="C73" t="s">
-        <v>1375</v>
+        <v>1373</v>
       </c>
       <c r="D73" t="s">
         <v>301</v>
@@ -5680,6 +5743,9 @@
       <c r="B74" t="s">
         <v>55</v>
       </c>
+      <c r="C74" t="s">
+        <v>1429</v>
+      </c>
       <c r="D74" t="s">
         <v>271</v>
       </c>
@@ -5750,7 +5816,7 @@
         <v>234</v>
       </c>
       <c r="C80" t="s">
-        <v>1309</v>
+        <v>1416</v>
       </c>
       <c r="D80" t="s">
         <v>291</v>
@@ -5775,7 +5841,7 @@
         <v>288</v>
       </c>
       <c r="C82" t="s">
-        <v>1402</v>
+        <v>1419</v>
       </c>
       <c r="D82" t="s">
         <v>289</v>
@@ -5788,6 +5854,9 @@
       <c r="B83" t="s">
         <v>71</v>
       </c>
+      <c r="C83" t="s">
+        <v>1417</v>
+      </c>
       <c r="D83" t="s">
         <v>289</v>
       </c>
@@ -5800,7 +5869,7 @@
         <v>204</v>
       </c>
       <c r="C84" t="s">
-        <v>1366</v>
+        <v>1437</v>
       </c>
       <c r="D84" t="s">
         <v>293</v>
@@ -5902,7 +5971,7 @@
         <v>83</v>
       </c>
       <c r="C93" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="D93" t="s">
         <v>273</v>
@@ -6004,7 +6073,7 @@
         <v>192</v>
       </c>
       <c r="C102" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="D102" t="s">
         <v>214</v>
@@ -6018,7 +6087,7 @@
         <v>105</v>
       </c>
       <c r="C103" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
       <c r="D103" t="s">
         <v>214</v>
@@ -6032,7 +6101,7 @@
         <v>171</v>
       </c>
       <c r="C104" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="D104" t="s">
         <v>225</v>
@@ -6074,7 +6143,7 @@
         <v>213</v>
       </c>
       <c r="C107" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="D107" t="s">
         <v>251</v>
@@ -6102,7 +6171,7 @@
         <v>102</v>
       </c>
       <c r="C109" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="D109" t="s">
         <v>211</v>
@@ -6163,7 +6232,7 @@
         <v>106</v>
       </c>
       <c r="C114" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="D114" t="s">
         <v>232</v>
@@ -6177,7 +6246,7 @@
         <v>189</v>
       </c>
       <c r="C115" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="D115" t="s">
         <v>236</v>
@@ -6219,7 +6288,7 @@
         <v>237</v>
       </c>
       <c r="C118" t="s">
-        <v>1328</v>
+        <v>1412</v>
       </c>
       <c r="D118" t="s">
         <v>235</v>
@@ -6277,7 +6346,7 @@
         <v>141</v>
       </c>
       <c r="C123" t="s">
-        <v>1395</v>
+        <v>1393</v>
       </c>
       <c r="D123" t="s">
         <v>269</v>
@@ -6291,7 +6360,7 @@
         <v>175</v>
       </c>
       <c r="C124" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="D124" t="s">
         <v>261</v>
@@ -6352,7 +6421,7 @@
         <v>182</v>
       </c>
       <c r="C129" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="D129" t="s">
         <v>248</v>
@@ -6388,7 +6457,7 @@
         <v>179</v>
       </c>
       <c r="C132" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="D132" t="s">
         <v>268</v>
@@ -6402,7 +6471,7 @@
         <v>240</v>
       </c>
       <c r="C133" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="D133" t="s">
         <v>247</v>
@@ -6429,6 +6498,9 @@
       <c r="B135" t="s">
         <v>99</v>
       </c>
+      <c r="C135" t="s">
+        <v>1433</v>
+      </c>
       <c r="D135" t="s">
         <v>287</v>
       </c>
@@ -6440,6 +6512,9 @@
       <c r="B136" t="s">
         <v>100</v>
       </c>
+      <c r="C136" t="s">
+        <v>1433</v>
+      </c>
       <c r="D136" t="s">
         <v>286</v>
       </c>
@@ -6451,6 +6526,9 @@
       <c r="B137" t="s">
         <v>40</v>
       </c>
+      <c r="C137" t="s">
+        <v>1429</v>
+      </c>
       <c r="D137" t="s">
         <v>250</v>
       </c>
@@ -6463,7 +6541,7 @@
         <v>243</v>
       </c>
       <c r="C138" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="D138" t="s">
         <v>290</v>
@@ -6477,7 +6555,7 @@
         <v>35</v>
       </c>
       <c r="C139" t="s">
-        <v>1309</v>
+        <v>1415</v>
       </c>
       <c r="D139" t="s">
         <v>263</v>
@@ -6491,7 +6569,7 @@
         <v>76</v>
       </c>
       <c r="C140" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
       <c r="D140" t="s">
         <v>297</v>
@@ -6505,7 +6583,7 @@
         <v>170</v>
       </c>
       <c r="C141" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="D141" t="s">
         <v>285</v>
@@ -6540,6 +6618,9 @@
       <c r="B144" t="s">
         <v>202</v>
       </c>
+      <c r="C144" t="s">
+        <v>1434</v>
+      </c>
       <c r="D144" t="s">
         <v>270</v>
       </c>
@@ -6650,6 +6731,9 @@
       <c r="B154" t="s">
         <v>82</v>
       </c>
+      <c r="C154" t="s">
+        <v>1417</v>
+      </c>
       <c r="D154" t="s">
         <v>294</v>
       </c>
@@ -6661,6 +6745,9 @@
       <c r="B155" t="s">
         <v>67</v>
       </c>
+      <c r="C155" t="s">
+        <v>1433</v>
+      </c>
       <c r="D155" t="s">
         <v>314</v>
       </c>
@@ -6716,6 +6803,9 @@
       <c r="B160" t="s">
         <v>238</v>
       </c>
+      <c r="C160" t="s">
+        <v>1413</v>
+      </c>
       <c r="D160" t="s">
         <v>272</v>
       </c>
@@ -6750,7 +6840,7 @@
         <v>28</v>
       </c>
       <c r="C163" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="D163" t="s">
         <v>302</v>
@@ -6778,7 +6868,7 @@
         <v>316</v>
       </c>
       <c r="C165" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D165" t="s">
         <v>318</v>
@@ -6792,7 +6882,7 @@
         <v>326</v>
       </c>
       <c r="C166" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="D166" t="s">
         <v>325</v>
@@ -6806,7 +6896,7 @@
         <v>328</v>
       </c>
       <c r="C167" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="D167" t="s">
         <v>325</v>
@@ -6820,7 +6910,7 @@
         <v>329</v>
       </c>
       <c r="C168" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D168" t="s">
         <v>325</v>
@@ -6834,7 +6924,7 @@
         <v>333</v>
       </c>
       <c r="C169" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D169" t="s">
         <v>325</v>
@@ -6848,7 +6938,7 @@
         <v>342</v>
       </c>
       <c r="C170" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D170" t="s">
         <v>325</v>
@@ -6862,7 +6952,7 @@
         <v>343</v>
       </c>
       <c r="C171" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D171" t="s">
         <v>325</v>
@@ -6996,7 +7086,7 @@
         <v>131</v>
       </c>
       <c r="C181" t="s">
-        <v>1295</v>
+        <v>1438</v>
       </c>
       <c r="D181" t="s">
         <v>217</v>
@@ -7024,7 +7114,7 @@
         <v>155</v>
       </c>
       <c r="C183" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="D183" t="s">
         <v>217</v>
@@ -7049,7 +7139,7 @@
         <v>152</v>
       </c>
       <c r="C185" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="D185" t="s">
         <v>217</v>
@@ -7063,7 +7153,7 @@
         <v>162</v>
       </c>
       <c r="C186" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="D186" t="s">
         <v>222</v>
@@ -7241,7 +7331,7 @@
         <v>380</v>
       </c>
       <c r="C206" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -7252,7 +7342,7 @@
         <v>381</v>
       </c>
       <c r="C207" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
@@ -7263,7 +7353,7 @@
         <v>383</v>
       </c>
       <c r="C208" t="s">
-        <v>1309</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
@@ -7282,7 +7372,7 @@
         <v>0</v>
       </c>
       <c r="C210" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
@@ -7301,7 +7391,7 @@
         <v>386</v>
       </c>
       <c r="C212" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
@@ -7312,7 +7402,7 @@
         <v>387</v>
       </c>
       <c r="C213" t="s">
-        <v>1409</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
@@ -7331,7 +7421,7 @@
         <v>389</v>
       </c>
       <c r="C215" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -7342,7 +7432,7 @@
         <v>390</v>
       </c>
       <c r="C216" t="s">
-        <v>1409</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
@@ -7380,7 +7470,7 @@
         <v>1</v>
       </c>
       <c r="C220" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
@@ -7418,7 +7508,7 @@
         <v>398</v>
       </c>
       <c r="C224" t="s">
-        <v>1415</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
@@ -7429,7 +7519,7 @@
         <v>399</v>
       </c>
       <c r="C225" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
@@ -7450,6 +7540,9 @@
       <c r="B227" t="s">
         <v>402</v>
       </c>
+      <c r="C227" t="s">
+        <v>1433</v>
+      </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
@@ -7502,7 +7595,7 @@
         <v>409</v>
       </c>
       <c r="C233" t="s">
-        <v>1411</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -7537,7 +7630,7 @@
         <v>413</v>
       </c>
       <c r="C237" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
@@ -7556,7 +7649,7 @@
         <v>415</v>
       </c>
       <c r="C239" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
@@ -7575,7 +7668,7 @@
         <v>418</v>
       </c>
       <c r="C241" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
@@ -7594,7 +7687,7 @@
         <v>420</v>
       </c>
       <c r="C243" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
@@ -7621,7 +7714,7 @@
         <v>424</v>
       </c>
       <c r="C246" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
@@ -7651,7 +7744,7 @@
         <v>427</v>
       </c>
       <c r="C249" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
@@ -7713,7 +7806,7 @@
         <v>433</v>
       </c>
       <c r="C256" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
@@ -7740,7 +7833,7 @@
         <v>435</v>
       </c>
       <c r="C259" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
@@ -7797,7 +7890,7 @@
         <v>440</v>
       </c>
       <c r="C265" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
@@ -7805,7 +7898,7 @@
         <v>797</v>
       </c>
       <c r="B266" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
@@ -7840,7 +7933,7 @@
         <v>445</v>
       </c>
       <c r="C270" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
@@ -7875,7 +7968,7 @@
         <v>449</v>
       </c>
       <c r="C274" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
@@ -7902,7 +7995,7 @@
         <v>452</v>
       </c>
       <c r="C277" t="s">
-        <v>1396</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
@@ -7932,7 +8025,7 @@
         <v>456</v>
       </c>
       <c r="C280" t="s">
-        <v>1373</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
@@ -7967,7 +8060,7 @@
         <v>460</v>
       </c>
       <c r="C284" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
@@ -7986,7 +8079,7 @@
         <v>462</v>
       </c>
       <c r="C286" t="s">
-        <v>1414</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
@@ -8005,7 +8098,7 @@
         <v>465</v>
       </c>
       <c r="C288" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
@@ -8016,7 +8109,7 @@
         <v>466</v>
       </c>
       <c r="C289" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
@@ -8059,7 +8152,7 @@
         <v>472</v>
       </c>
       <c r="C294" t="s">
-        <v>1396</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
@@ -8094,7 +8187,7 @@
         <v>480</v>
       </c>
       <c r="C298" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
@@ -8104,6 +8197,9 @@
       <c r="B299" t="s">
         <v>481</v>
       </c>
+      <c r="C299" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
@@ -8137,7 +8233,7 @@
         <v>8</v>
       </c>
       <c r="C303" t="s">
-        <v>1321</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
@@ -8156,7 +8252,7 @@
         <v>487</v>
       </c>
       <c r="C305" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -8167,7 +8263,7 @@
         <v>489</v>
       </c>
       <c r="C306" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
@@ -8177,6 +8273,9 @@
       <c r="B307" t="s">
         <v>493</v>
       </c>
+      <c r="C307" t="s">
+        <v>1429</v>
+      </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
@@ -8194,7 +8293,7 @@
         <v>10</v>
       </c>
       <c r="C309" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
@@ -8293,7 +8392,7 @@
         <v>515</v>
       </c>
       <c r="C321" t="s">
-        <v>1411</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
@@ -8312,7 +8411,7 @@
         <v>517</v>
       </c>
       <c r="C323" t="s">
-        <v>1399</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
@@ -8331,7 +8430,7 @@
         <v>519</v>
       </c>
       <c r="C325" t="s">
-        <v>1403</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
@@ -8478,7 +8577,7 @@
         <v>50</v>
       </c>
       <c r="C343" t="s">
-        <v>1416</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
@@ -8496,6 +8595,9 @@
       <c r="B345" t="s">
         <v>245</v>
       </c>
+      <c r="C345" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
@@ -8553,7 +8655,7 @@
         <v>12</v>
       </c>
       <c r="C352" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.25">
@@ -8572,7 +8674,7 @@
         <v>538</v>
       </c>
       <c r="C354" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.25">
@@ -8607,7 +8709,7 @@
         <v>543</v>
       </c>
       <c r="C358" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.25">
@@ -8634,7 +8736,7 @@
         <v>547</v>
       </c>
       <c r="C361" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
@@ -8669,7 +8771,7 @@
         <v>549</v>
       </c>
       <c r="C365" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
@@ -8696,7 +8798,7 @@
         <v>554</v>
       </c>
       <c r="C368" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.25">
@@ -8707,7 +8809,7 @@
         <v>556</v>
       </c>
       <c r="C369" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.25">
@@ -8734,7 +8836,7 @@
         <v>559</v>
       </c>
       <c r="C372" t="s">
-        <v>1414</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.25">
@@ -8788,7 +8890,7 @@
         <v>565</v>
       </c>
       <c r="C378" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="379" spans="1:3" x14ac:dyDescent="0.25">
@@ -8799,7 +8901,7 @@
         <v>566</v>
       </c>
       <c r="C379" t="s">
-        <v>1382</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.25">
@@ -8809,6 +8911,9 @@
       <c r="B380" t="s">
         <v>16</v>
       </c>
+      <c r="C380" t="s">
+        <v>1433</v>
+      </c>
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
@@ -8837,7 +8942,7 @@
         <v>572</v>
       </c>
       <c r="C383" t="s">
-        <v>1401</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.25">
@@ -8855,6 +8960,9 @@
       <c r="B385" t="s">
         <v>574</v>
       </c>
+      <c r="C385" t="s">
+        <v>1429</v>
+      </c>
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
@@ -8871,6 +8979,9 @@
       <c r="B387" t="s">
         <v>577</v>
       </c>
+      <c r="C387" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
@@ -8879,6 +8990,9 @@
       <c r="B388" t="s">
         <v>17</v>
       </c>
+      <c r="C388" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="389" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
@@ -8903,6 +9017,9 @@
       <c r="B391" t="s">
         <v>19</v>
       </c>
+      <c r="C391" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
@@ -8955,7 +9072,7 @@
         <v>464</v>
       </c>
       <c r="C397" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.25">
@@ -8966,7 +9083,7 @@
         <v>467</v>
       </c>
       <c r="C398" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.25">
@@ -9181,7 +9298,7 @@
         <v>603</v>
       </c>
       <c r="C423" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.25">
@@ -9200,7 +9317,7 @@
         <v>605</v>
       </c>
       <c r="C425" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.25">
@@ -9219,7 +9336,7 @@
         <v>104</v>
       </c>
       <c r="C427" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="428" spans="1:3" x14ac:dyDescent="0.25">
@@ -9316,7 +9433,7 @@
         <v>615</v>
       </c>
       <c r="C438" t="s">
-        <v>1381</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.25">
@@ -9343,7 +9460,7 @@
         <v>617</v>
       </c>
       <c r="C441" t="s">
-        <v>1411</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
@@ -9389,7 +9506,7 @@
         <v>622</v>
       </c>
       <c r="C446" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
@@ -9502,7 +9619,7 @@
         <v>635</v>
       </c>
       <c r="C459" t="s">
-        <v>1412</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.25">
@@ -9545,7 +9662,7 @@
         <v>640</v>
       </c>
       <c r="C464" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
@@ -9564,7 +9681,7 @@
         <v>642</v>
       </c>
       <c r="C466" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
@@ -9575,7 +9692,7 @@
         <v>643</v>
       </c>
       <c r="C467" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
@@ -9586,7 +9703,7 @@
         <v>644</v>
       </c>
       <c r="C468" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
@@ -9597,7 +9714,7 @@
         <v>645</v>
       </c>
       <c r="C469" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="470" spans="1:3" x14ac:dyDescent="0.25">
@@ -9627,7 +9744,7 @@
         <v>648</v>
       </c>
       <c r="C472" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
@@ -9646,7 +9763,7 @@
         <v>650</v>
       </c>
       <c r="C474" t="s">
-        <v>1413</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
@@ -9696,6 +9813,9 @@
       <c r="B480" t="s">
         <v>656</v>
       </c>
+      <c r="C480" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
@@ -9720,6 +9840,9 @@
       <c r="B483" t="s">
         <v>658</v>
       </c>
+      <c r="C483" t="s">
+        <v>1417</v>
+      </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
@@ -9758,6 +9881,9 @@
       <c r="B487" t="s">
         <v>661</v>
       </c>
+      <c r="C487" t="s">
+        <v>1429</v>
+      </c>
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
@@ -9774,6 +9900,9 @@
       <c r="B489" t="s">
         <v>664</v>
       </c>
+      <c r="C489" t="s">
+        <v>1434</v>
+      </c>
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
@@ -9806,6 +9935,9 @@
       <c r="B493" t="s">
         <v>173</v>
       </c>
+      <c r="C493" t="s">
+        <v>1423</v>
+      </c>
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
@@ -9887,7 +10019,7 @@
         <v>674</v>
       </c>
       <c r="C503" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
@@ -10026,7 +10158,7 @@
         <v>136</v>
       </c>
       <c r="C520" t="s">
-        <v>1410</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
@@ -10045,7 +10177,7 @@
         <v>107</v>
       </c>
       <c r="C522" t="s">
-        <v>1332</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
@@ -10393,7 +10525,7 @@
         <v>153</v>
       </c>
       <c r="C564" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="565" spans="1:3" x14ac:dyDescent="0.25">
@@ -10428,7 +10560,7 @@
         <v>79</v>
       </c>
       <c r="C568" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="569" spans="1:3" x14ac:dyDescent="0.25">
@@ -10546,7 +10678,7 @@
         <v>65</v>
       </c>
       <c r="C582" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="583" spans="1:3" x14ac:dyDescent="0.25">
@@ -10557,7 +10689,7 @@
         <v>66</v>
       </c>
       <c r="C583" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="584" spans="1:3" x14ac:dyDescent="0.25">
@@ -10802,7 +10934,7 @@
     </row>
     <row r="614" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B614" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="C614" t="s">
         <v>1295</v>
@@ -10810,7 +10942,7 @@
     </row>
     <row r="615" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B615" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="C615" t="s">
         <v>1294</v>
@@ -10818,108 +10950,129 @@
     </row>
     <row r="616" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B616" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="617" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B617" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
       <c r="C617" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="618" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B618" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="619" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B619" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="C619" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="620" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B620" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="621" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B621" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="C621" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="622" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B622" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="623" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B623" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="C623" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="624" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B624" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="625" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B625" t="s">
-        <v>1387</v>
+        <v>1385</v>
       </c>
       <c r="C625" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="626" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B626" t="s">
-        <v>1388</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="627" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B627" t="s">
-        <v>1389</v>
+        <v>1387</v>
+      </c>
+      <c r="C627" t="s">
+        <v>1417</v>
       </c>
     </row>
     <row r="628" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B628" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="629" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B629" t="s">
-        <v>1391</v>
+        <v>1389</v>
       </c>
       <c r="C629" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="630" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B630" t="s">
-        <v>1392</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="631" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B631" t="s">
-        <v>1393</v>
+        <v>1391</v>
       </c>
       <c r="C631" t="s">
-        <v>1408</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="632" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B632" t="s">
-        <v>1394</v>
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="633" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B633" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="634" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B634" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C634" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="635" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B635" t="s">
+        <v>1428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>